<commit_message>
feat: implement comprehensive reporting system with Excel and PDF export capabilities for portfolio, delinquent, and receipt data
</commit_message>
<xml_diff>
--- a/Cooperativa_Resumen_Pagos_2026-04-07.xlsx
+++ b/Cooperativa_Resumen_Pagos_2026-04-07.xlsx
@@ -1,26 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3BFF59-0C11-4EB4-B358-36D2F16F993A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Resumen Pagos" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Resumen Pagos" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="70">
   <si>
     <t xml:space="preserve">  Resumen de Pagos - Boletas</t>
   </si>
   <si>
-    <t>Generado el: 6/4/2026 a las 6:30:54 p. m.</t>
+    <t>Generado el: 6/4/2026 a las 8:08:50 p. m.</t>
   </si>
   <si>
     <t>CLIENTE: Aldo Rene Castillo Cifuentes</t>
@@ -230,62 +226,52 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="10" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <color rgb="2563EB"/>
       <sz val="10"/>
-      <color rgb="FF2563EB"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -297,27 +283,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2563EB"/>
+        <fgColor rgb="2563EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3F4F6"/>
+        <fgColor rgb="F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E3A5F"/>
+        <fgColor rgb="1E3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF3B82F6"/>
+        <fgColor rgb="3B82F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF059669"/>
+        <fgColor rgb="059669"/>
       </patternFill>
     </fill>
   </fills>
@@ -330,32 +316,24 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="E5E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="E5E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="E5E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE5E7EB"/>
+        <color rgb="E5E7EB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -365,6 +343,15 @@
   </cellStyleXfs>
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -377,19 +364,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,17 +387,17 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1354666" cy="609600"/>
+    <xdr:ext cx="952500" cy="428625"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="1" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
@@ -439,7 +417,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="1354666" cy="609600"/>
+          <a:ext cx="0" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -772,994 +750,1006 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C103"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C104"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" ht="50" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-    </row>
-    <row r="4" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="4" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="A6" s="5">
         <v>1</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+    <row r="7" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="A9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+      <c r="A10" s="5">
         <v>1</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+    <row r="11" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="A13" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+      <c r="A14" s="5">
         <v>1</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="B14" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+      <c r="A15" s="5">
         <v>2</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
-        <v>3</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="4" t="s">
+      <c r="A16" s="5">
+        <v>3</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
-        <v>4</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="A17" s="5">
+        <v>4</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="A18" s="5">
         <v>5</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="B18" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
-        <v>6</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="A19" s="5">
+        <v>6</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="A20" s="5">
         <v>7</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="4" t="s">
+      <c r="B20" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+      <c r="A21" s="5">
         <v>8</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+      <c r="A22" s="5">
         <v>1</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C22" s="4" t="s">
+      <c r="B22" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
+    <row r="23" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="A25" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+      <c r="A26" s="5">
         <v>1</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C26" s="4" t="s">
+      <c r="B26" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
+    <row r="27" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C29" s="1" t="s">
+      <c r="A29" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+      <c r="A30" s="5">
         <v>1</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="4" t="s">
+      <c r="B30" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="7" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+      <c r="A31" s="5">
         <v>2</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" s="4" t="s">
+      <c r="B31" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
-        <v>3</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" s="4" t="s">
+      <c r="A32" s="5">
+        <v>3</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="s">
+    <row r="33" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C35" s="1" t="s">
+      <c r="A35" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+      <c r="A36" s="5">
         <v>1</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" s="4" t="s">
+      <c r="B36" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="8" t="s">
+    <row r="37" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="A39" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+      <c r="A40" s="5">
         <v>1</v>
       </c>
-      <c r="B40" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40" s="4" t="s">
+      <c r="B40" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+      <c r="A41" s="5">
         <v>2</v>
       </c>
-      <c r="B41" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="4" t="s">
+      <c r="B41" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
-        <v>3</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" s="4" t="s">
+      <c r="A42" s="5">
+        <v>3</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
-        <v>4</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" s="4" t="s">
+      <c r="A43" s="5">
+        <v>4</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+      <c r="A44" s="5">
         <v>5</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="4" t="s">
+      <c r="B44" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
-        <v>6</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" s="4" t="s">
+      <c r="A45" s="5">
+        <v>6</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="8" t="s">
+    <row r="46" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C48" s="1" t="s">
+      <c r="A48" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+      <c r="A49" s="5">
         <v>1</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C49" s="4" t="s">
+      <c r="B49" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+      <c r="A50" s="5">
         <v>2</v>
       </c>
-      <c r="B50" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C50" s="4" t="s">
+      <c r="B50" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" s="7" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
-        <v>3</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C51" s="4" t="s">
+      <c r="A51" s="5">
+        <v>3</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" s="7" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
-        <v>4</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C52" s="4" t="s">
+      <c r="A52" s="5">
+        <v>4</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
+      <c r="A53" s="5">
         <v>5</v>
       </c>
-      <c r="B53" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C53" s="4" t="s">
+      <c r="B53" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C53" s="7" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
-        <v>6</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C54" s="4" t="s">
+      <c r="A54" s="5">
+        <v>6</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C54" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
+      <c r="A55" s="5">
         <v>7</v>
       </c>
-      <c r="B55" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C55" s="4" t="s">
+      <c r="B55" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C55" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
+      <c r="A56" s="5">
         <v>8</v>
       </c>
-      <c r="B56" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C56" s="4" t="s">
+      <c r="B56" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C56" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
+      <c r="A57" s="5">
         <v>1</v>
       </c>
-      <c r="B57" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C57" s="4" t="s">
+      <c r="B57" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" s="7" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
+      <c r="A58" s="5">
         <v>2</v>
       </c>
-      <c r="B58" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C58" s="4" t="s">
+      <c r="B58" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" s="7" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
-        <v>3</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C59" s="4" t="s">
+      <c r="A59" s="5">
+        <v>3</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
-        <v>4</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C60" s="4" t="s">
+      <c r="A60" s="5">
+        <v>4</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" s="7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
+      <c r="A61" s="5">
         <v>5</v>
       </c>
-      <c r="B61" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C61" s="4" t="s">
+      <c r="B61" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" s="7" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="2">
-        <v>6</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C62" s="4" t="s">
+      <c r="A62" s="5">
+        <v>6</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C62" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="2">
+      <c r="A63" s="5">
         <v>7</v>
       </c>
-      <c r="B63" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C63" s="4" t="s">
+      <c r="B63" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C63" s="7" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="2">
+      <c r="A64" s="5">
         <v>8</v>
       </c>
-      <c r="B64" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C64" s="4" t="s">
+      <c r="B64" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C64" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="8" t="s">
+    <row r="65" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B66" s="8"/>
-      <c r="C66" s="8"/>
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C67" s="1" t="s">
+      <c r="A67" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" s="2">
+      <c r="A68" s="5">
         <v>1</v>
       </c>
-      <c r="B68" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C68" s="4" t="s">
+      <c r="B68" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C68" s="7" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" s="2">
+      <c r="A69" s="5">
         <v>2</v>
       </c>
-      <c r="B69" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C69" s="4" t="s">
+      <c r="B69" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" s="7" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="8" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="5">
+        <v>3</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="71" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B71" s="8"/>
-      <c r="C71" s="8"/>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C72" s="1" t="s">
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" s="2">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="5">
         <v>1</v>
       </c>
-      <c r="B73" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C73" s="4" t="s">
+      <c r="B74" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C74" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" s="2">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="5">
         <v>2</v>
       </c>
-      <c r="B74" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C74" s="4" t="s">
+      <c r="B75" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C75" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" s="2">
-        <v>3</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C75" s="4" t="s">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="5">
+        <v>3</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C76" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="8" t="s">
+    <row r="77" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B77" s="8"/>
-      <c r="C77" s="8"/>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C78" s="1" t="s">
+      <c r="B78" s="3"/>
+      <c r="C78" s="3"/>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" s="2">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="5">
         <v>1</v>
       </c>
-      <c r="B79" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C79" s="4" t="s">
+      <c r="B80" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C80" s="7" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="8" t="s">
+    <row r="81" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="82" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B81" s="8"/>
-      <c r="C81" s="8"/>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C82" s="1" t="s">
+      <c r="B82" s="3"/>
+      <c r="C82" s="3"/>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A83" s="2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="5">
         <v>1</v>
       </c>
-      <c r="B83" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C83" s="4" t="s">
+      <c r="B84" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C84" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="8" t="s">
+    <row r="85" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B85" s="8"/>
-      <c r="C85" s="8"/>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C86" s="1" t="s">
+      <c r="B86" s="3"/>
+      <c r="C86" s="3"/>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="2">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="5">
         <v>1</v>
       </c>
-      <c r="B87" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C87" s="4" t="s">
+      <c r="B88" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C88" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A88" s="2">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="5">
         <v>2</v>
       </c>
-      <c r="B88" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C88" s="4" t="s">
+      <c r="B89" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C89" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A89" s="2">
-        <v>3</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C89" s="4" t="s">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="5">
+        <v>3</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A90" s="2">
-        <v>4</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C90" s="4" t="s">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="5">
+        <v>4</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C91" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91" s="2">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="5">
         <v>5</v>
       </c>
-      <c r="B91" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C91" s="4" t="s">
+      <c r="B92" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C92" s="7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A92" s="2">
-        <v>6</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C92" s="4" t="s">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="5">
+        <v>6</v>
+      </c>
+      <c r="B93" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C93" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="24" x14ac:dyDescent="0.25">
-      <c r="A93" s="2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="5">
         <v>7</v>
       </c>
-      <c r="B93" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C93" s="4" t="s">
+      <c r="B94" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C94" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A94" s="2">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="5">
         <v>1</v>
       </c>
-      <c r="B94" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C94" s="4" t="s">
+      <c r="B95" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C95" s="7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A95" s="2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="5">
         <v>2</v>
       </c>
-      <c r="B95" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C95" s="4" t="s">
+      <c r="B96" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C96" s="7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A96" s="2">
-        <v>3</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C96" s="4" t="s">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" s="5">
+        <v>3</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C97" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A97" s="2">
-        <v>4</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C97" s="4" t="s">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="5">
+        <v>4</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C98" s="7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A100" s="9" t="s">
+    <row r="99" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="B100" s="9"/>
-      <c r="C100" s="9"/>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A102" s="5" t="s">
+      <c r="B101" s="8"/>
+      <c r="C101" s="8"/>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B102">
+      <c r="B103">
         <v>13</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A103" s="5" t="s">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B103">
-        <v>56</v>
+      <c r="B104">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A100:C100"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A71:C71"/>
-    <mergeCell ref="A77:C77"/>
-    <mergeCell ref="A81:C81"/>
-    <mergeCell ref="A85:C85"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="A47:C47"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A66:C66"/>
+    <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A78:C78"/>
+    <mergeCell ref="A82:C82"/>
+    <mergeCell ref="A86:C86"/>
+    <mergeCell ref="A101:C101"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B10" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B14" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="B15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="B16" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B17" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B18" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="B19" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="B20" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="B21" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="B22" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="B26" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="B30" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="B31" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="B32" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="B36" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B40" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B41" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B42" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B43" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B44" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="B45" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="B49" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="B50" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="B51" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="B52" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="B53" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="B54" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="B55" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="B56" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="B57" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="B58" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="B59" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="B60" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="B61" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="B62" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="B63" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="B64" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="B68" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="B69" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="B73" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="B74" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="B75" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="B79" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="B83" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="B87" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="B88" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="B89" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="B90" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="B91" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="B92" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="B93" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="B94" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="B95" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="B96" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="B97" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="B6" r:id="rId1"/>
+    <hyperlink ref="B10" r:id="rId2"/>
+    <hyperlink ref="B14" r:id="rId3"/>
+    <hyperlink ref="B15" r:id="rId4"/>
+    <hyperlink ref="B16" r:id="rId5"/>
+    <hyperlink ref="B17" r:id="rId6"/>
+    <hyperlink ref="B18" r:id="rId7"/>
+    <hyperlink ref="B19" r:id="rId8"/>
+    <hyperlink ref="B20" r:id="rId9"/>
+    <hyperlink ref="B21" r:id="rId10"/>
+    <hyperlink ref="B22" r:id="rId11"/>
+    <hyperlink ref="B26" r:id="rId12"/>
+    <hyperlink ref="B30" r:id="rId13"/>
+    <hyperlink ref="B31" r:id="rId14"/>
+    <hyperlink ref="B32" r:id="rId15"/>
+    <hyperlink ref="B36" r:id="rId16"/>
+    <hyperlink ref="B40" r:id="rId17"/>
+    <hyperlink ref="B41" r:id="rId18"/>
+    <hyperlink ref="B42" r:id="rId19"/>
+    <hyperlink ref="B43" r:id="rId20"/>
+    <hyperlink ref="B44" r:id="rId21"/>
+    <hyperlink ref="B45" r:id="rId22"/>
+    <hyperlink ref="B49" r:id="rId23"/>
+    <hyperlink ref="B50" r:id="rId24"/>
+    <hyperlink ref="B51" r:id="rId25"/>
+    <hyperlink ref="B52" r:id="rId26"/>
+    <hyperlink ref="B53" r:id="rId27"/>
+    <hyperlink ref="B54" r:id="rId28"/>
+    <hyperlink ref="B55" r:id="rId29"/>
+    <hyperlink ref="B56" r:id="rId30"/>
+    <hyperlink ref="B57" r:id="rId31"/>
+    <hyperlink ref="B58" r:id="rId32"/>
+    <hyperlink ref="B59" r:id="rId33"/>
+    <hyperlink ref="B60" r:id="rId34"/>
+    <hyperlink ref="B61" r:id="rId35"/>
+    <hyperlink ref="B62" r:id="rId36"/>
+    <hyperlink ref="B63" r:id="rId37"/>
+    <hyperlink ref="B64" r:id="rId38"/>
+    <hyperlink ref="B68" r:id="rId39"/>
+    <hyperlink ref="B69" r:id="rId40"/>
+    <hyperlink ref="B70" r:id="rId41"/>
+    <hyperlink ref="B74" r:id="rId42"/>
+    <hyperlink ref="B75" r:id="rId43"/>
+    <hyperlink ref="B76" r:id="rId44"/>
+    <hyperlink ref="B80" r:id="rId45"/>
+    <hyperlink ref="B84" r:id="rId46"/>
+    <hyperlink ref="B88" r:id="rId47"/>
+    <hyperlink ref="B89" r:id="rId48"/>
+    <hyperlink ref="B90" r:id="rId49"/>
+    <hyperlink ref="B91" r:id="rId50"/>
+    <hyperlink ref="B92" r:id="rId51"/>
+    <hyperlink ref="B93" r:id="rId52"/>
+    <hyperlink ref="B94" r:id="rId53"/>
+    <hyperlink ref="B95" r:id="rId54"/>
+    <hyperlink ref="B96" r:id="rId55"/>
+    <hyperlink ref="B97" r:id="rId56"/>
+    <hyperlink ref="B98" r:id="rId57"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <drawing r:id="rId57"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId58"/>
 </worksheet>
 </file>
</xml_diff>